<commit_message>
EPBDS-15833 Fix code review
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/Math.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/Math.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vpikus/Sources/OpenL/openl-tablets/DEV/org.openl.rules.test/test-resources/functionality/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4862A5FF-7075-6044-84E6-F3CB071E196C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498FC6F4-D6ED-FF48-9CE4-2075399052DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="780" windowWidth="34980" windowHeight="22600" tabRatio="765" firstSheet="5" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2238,15 +2238,6 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="21" fillId="10" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2265,6 +2256,15 @@
     <xf numFmtId="0" fontId="10" fillId="7" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2279,9 +2279,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2306,6 +2303,9 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3103,28 +3103,28 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:5" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B2" s="81" t="s">
+      <c r="B2" s="78" t="s">
         <v>282</v>
       </c>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
+      <c r="C2" s="79"/>
+      <c r="D2" s="79"/>
+      <c r="E2" s="79"/>
     </row>
     <row r="3" spans="2:5" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B3" s="83" t="s">
+      <c r="B3" s="80" t="s">
         <v>283</v>
       </c>
-      <c r="C3" s="84"/>
-      <c r="D3" s="84"/>
-      <c r="E3" s="84"/>
+      <c r="C3" s="81"/>
+      <c r="D3" s="81"/>
+      <c r="E3" s="81"/>
     </row>
     <row r="5" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B5" s="85" t="s">
+      <c r="B5" s="82" t="s">
         <v>284</v>
       </c>
-      <c r="C5" s="86"/>
-      <c r="D5" s="86"/>
-      <c r="E5" s="86"/>
+      <c r="C5" s="83"/>
+      <c r="D5" s="83"/>
+      <c r="E5" s="83"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B6" s="47" t="s">
@@ -3331,28 +3331,28 @@
       <c r="E21" s="50"/>
     </row>
     <row r="25" spans="2:5" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B25" s="81" t="s">
+      <c r="B25" s="78" t="s">
         <v>278</v>
       </c>
-      <c r="C25" s="82"/>
-      <c r="D25" s="82"/>
-      <c r="E25" s="82"/>
+      <c r="C25" s="79"/>
+      <c r="D25" s="79"/>
+      <c r="E25" s="79"/>
     </row>
     <row r="26" spans="2:5" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B26" s="83" t="s">
+      <c r="B26" s="80" t="s">
         <v>280</v>
       </c>
-      <c r="C26" s="84"/>
-      <c r="D26" s="84"/>
-      <c r="E26" s="84"/>
+      <c r="C26" s="81"/>
+      <c r="D26" s="81"/>
+      <c r="E26" s="81"/>
     </row>
     <row r="28" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B28" s="85" t="s">
+      <c r="B28" s="82" t="s">
         <v>277</v>
       </c>
-      <c r="C28" s="86"/>
-      <c r="D28" s="86"/>
-      <c r="E28" s="86"/>
+      <c r="C28" s="83"/>
+      <c r="D28" s="83"/>
+      <c r="E28" s="83"/>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B29" s="47" t="s">
@@ -6672,7 +6672,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{371F3650-624E-7A4C-9A5A-E52222BCB235}">
-  <dimension ref="B5:E161"/>
+  <dimension ref="B5:E159"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="2" max="2" width="20.6640625" customWidth="1"/>
@@ -6682,20 +6682,20 @@
   </cols>
   <sheetData>
     <row r="5" spans="2:5" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B5" s="81" t="s">
+      <c r="B5" s="78" t="s">
         <v>340</v>
       </c>
-      <c r="C5" s="82"/>
-      <c r="D5" s="82"/>
-      <c r="E5" s="82"/>
+      <c r="C5" s="79"/>
+      <c r="D5" s="79"/>
+      <c r="E5" s="79"/>
     </row>
     <row r="6" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B6" s="83" t="s">
+      <c r="B6" s="80" t="s">
         <v>324</v>
       </c>
-      <c r="C6" s="84"/>
-      <c r="D6" s="84"/>
-      <c r="E6" s="84"/>
+      <c r="C6" s="81"/>
+      <c r="D6" s="81"/>
+      <c r="E6" s="81"/>
     </row>
     <row r="7" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B7" s="68"/>
@@ -6704,12 +6704,12 @@
       <c r="E7" s="68"/>
     </row>
     <row r="8" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B8" s="85" t="s">
+      <c r="B8" s="82" t="s">
         <v>325</v>
       </c>
-      <c r="C8" s="86"/>
-      <c r="D8" s="86"/>
-      <c r="E8" s="86"/>
+      <c r="C8" s="83"/>
+      <c r="D8" s="83"/>
+      <c r="E8" s="83"/>
     </row>
     <row r="9" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B9" s="47" t="s">
@@ -6886,52 +6886,52 @@
       <c r="E21" s="69"/>
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B22" s="50">
-        <v>12</v>
-      </c>
-      <c r="C22" s="50">
-        <v>-128</v>
-      </c>
-      <c r="D22" s="50">
-        <v>-1</v>
-      </c>
-      <c r="E22" s="50">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B23" s="75"/>
-      <c r="C23" s="75"/>
-      <c r="D23" s="75"/>
-      <c r="E23" s="75"/>
+      <c r="B22" s="75"/>
+      <c r="C22" s="75"/>
+      <c r="D22" s="75"/>
+      <c r="E22" s="75"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B25" s="84" t="s">
+        <v>341</v>
+      </c>
+      <c r="C25" s="84"/>
+      <c r="D25" s="84"/>
+      <c r="E25" s="84"/>
     </row>
     <row r="26" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B26" s="79" t="s">
-        <v>341</v>
-      </c>
-      <c r="C26" s="79"/>
-      <c r="D26" s="79"/>
-      <c r="E26" s="79"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B27" s="80" t="s">
+      <c r="B26" s="85" t="s">
         <v>324</v>
       </c>
-      <c r="C27" s="80"/>
-      <c r="D27" s="80"/>
-      <c r="E27" s="80"/>
+      <c r="C26" s="85"/>
+      <c r="D26" s="85"/>
+      <c r="E26" s="85"/>
+    </row>
+    <row r="28" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B28" s="86" t="s">
+        <v>326</v>
+      </c>
+      <c r="C28" s="86"/>
+      <c r="D28" s="86"/>
+      <c r="E28" s="86"/>
     </row>
     <row r="29" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B29" s="78" t="s">
-        <v>326</v>
-      </c>
-      <c r="C29" s="78"/>
-      <c r="D29" s="78"/>
-      <c r="E29" s="78"/>
+      <c r="B29" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C29" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D29" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E29" s="71" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B30" s="71" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C30" s="71" t="s">
         <v>321</v>
@@ -6940,1371 +6940,1343 @@
         <v>281</v>
       </c>
       <c r="E30" s="71" t="s">
-        <v>0</v>
+        <v>322</v>
       </c>
     </row>
     <row r="31" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B31" s="71" t="s">
+      <c r="B31" s="69">
+        <v>1</v>
+      </c>
+      <c r="C31" s="69">
+        <v>7</v>
+      </c>
+      <c r="D31" s="69">
+        <v>3</v>
+      </c>
+      <c r="E31" s="69">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="32" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B32" s="70">
+        <v>2</v>
+      </c>
+      <c r="C32" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D32" s="70">
+        <v>3</v>
+      </c>
+      <c r="E32" s="70">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="33" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B33" s="69">
+        <v>3</v>
+      </c>
+      <c r="C33" s="69">
+        <v>7</v>
+      </c>
+      <c r="D33" s="69">
+        <v>-3</v>
+      </c>
+      <c r="E33" s="69">
+        <v>-3</v>
+      </c>
+    </row>
+    <row r="34" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B34" s="70">
+        <v>4</v>
+      </c>
+      <c r="C34" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D34" s="70">
+        <v>-3</v>
+      </c>
+      <c r="E34" s="70">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="35" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B35" s="69">
+        <v>5</v>
+      </c>
+      <c r="C35" s="69">
+        <v>0</v>
+      </c>
+      <c r="D35" s="69">
+        <v>123</v>
+      </c>
+      <c r="E35" s="69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B36" s="70">
+        <v>6</v>
+      </c>
+      <c r="C36" s="70">
+        <v>32767</v>
+      </c>
+      <c r="D36" s="70">
+        <v>2</v>
+      </c>
+      <c r="E36" s="70">
+        <v>16383</v>
+      </c>
+    </row>
+    <row r="37" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B37" s="69">
+        <v>7</v>
+      </c>
+      <c r="C37" s="69">
+        <v>-32768</v>
+      </c>
+      <c r="D37" s="69">
+        <v>2</v>
+      </c>
+      <c r="E37" s="69">
+        <v>-16384</v>
+      </c>
+    </row>
+    <row r="38" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B38" s="70">
+        <v>8</v>
+      </c>
+      <c r="C38" s="70">
+        <v>-32767</v>
+      </c>
+      <c r="D38" s="70">
+        <v>2</v>
+      </c>
+      <c r="E38" s="70">
+        <v>-16384</v>
+      </c>
+    </row>
+    <row r="39" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B39" s="69">
+        <v>9</v>
+      </c>
+      <c r="C39" s="69">
+        <v>32767</v>
+      </c>
+      <c r="D39" s="69">
+        <v>-2</v>
+      </c>
+      <c r="E39" s="69">
+        <v>-16384</v>
+      </c>
+    </row>
+    <row r="40" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B40" s="50">
+        <v>10</v>
+      </c>
+      <c r="C40" s="50">
+        <v>7</v>
+      </c>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+    </row>
+    <row r="41" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B41" s="69">
+        <v>11</v>
+      </c>
+      <c r="C41" s="69"/>
+      <c r="D41" s="69">
+        <v>7</v>
+      </c>
+      <c r="E41" s="69"/>
+    </row>
+    <row r="42" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B42" s="75"/>
+      <c r="C42" s="75"/>
+      <c r="D42" s="75"/>
+      <c r="E42" s="75"/>
+    </row>
+    <row r="45" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B45" s="84" t="s">
+        <v>327</v>
+      </c>
+      <c r="C45" s="84"/>
+      <c r="D45" s="84"/>
+      <c r="E45" s="84"/>
+    </row>
+    <row r="46" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B46" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C46" s="85"/>
+      <c r="D46" s="85"/>
+      <c r="E46" s="85"/>
+    </row>
+    <row r="48" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B48" s="86" t="s">
+        <v>328</v>
+      </c>
+      <c r="C48" s="86"/>
+      <c r="D48" s="86"/>
+      <c r="E48" s="86"/>
+    </row>
+    <row r="49" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B49" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C49" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D49" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E49" s="71" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B50" s="71" t="s">
         <v>323</v>
       </c>
-      <c r="C31" s="71" t="s">
+      <c r="C50" s="71" t="s">
         <v>321</v>
       </c>
-      <c r="D31" s="71" t="s">
+      <c r="D50" s="71" t="s">
         <v>281</v>
       </c>
-      <c r="E31" s="71" t="s">
+      <c r="E50" s="71" t="s">
         <v>322</v>
       </c>
     </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B32" s="69">
-        <v>1</v>
-      </c>
-      <c r="C32" s="69">
+    <row r="51" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B51" s="69">
+        <v>1</v>
+      </c>
+      <c r="C51" s="69">
         <v>7</v>
       </c>
-      <c r="D32" s="69">
+      <c r="D51" s="69">
         <v>3</v>
       </c>
-      <c r="E32" s="69">
+      <c r="E51" s="69">
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B33" s="70">
+    <row r="52" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B52" s="70">
         <v>2</v>
       </c>
-      <c r="C33" s="70">
+      <c r="C52" s="70">
         <v>-7</v>
       </c>
-      <c r="D33" s="70">
+      <c r="D52" s="70">
         <v>3</v>
       </c>
-      <c r="E33" s="70">
+      <c r="E52" s="70">
         <v>-3</v>
-      </c>
-    </row>
-    <row r="34" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B34" s="69">
-        <v>3</v>
-      </c>
-      <c r="C34" s="69">
-        <v>7</v>
-      </c>
-      <c r="D34" s="69">
-        <v>-3</v>
-      </c>
-      <c r="E34" s="69">
-        <v>-3</v>
-      </c>
-    </row>
-    <row r="35" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B35" s="70">
-        <v>4</v>
-      </c>
-      <c r="C35" s="70">
-        <v>-7</v>
-      </c>
-      <c r="D35" s="70">
-        <v>-3</v>
-      </c>
-      <c r="E35" s="70">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="36" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B36" s="69">
-        <v>5</v>
-      </c>
-      <c r="C36" s="69">
-        <v>0</v>
-      </c>
-      <c r="D36" s="69">
-        <v>123</v>
-      </c>
-      <c r="E36" s="69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B37" s="70">
-        <v>6</v>
-      </c>
-      <c r="C37" s="70">
-        <v>32767</v>
-      </c>
-      <c r="D37" s="70">
-        <v>2</v>
-      </c>
-      <c r="E37" s="70">
-        <v>16383</v>
-      </c>
-    </row>
-    <row r="38" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B38" s="69">
-        <v>7</v>
-      </c>
-      <c r="C38" s="69">
-        <v>-32768</v>
-      </c>
-      <c r="D38" s="69">
-        <v>2</v>
-      </c>
-      <c r="E38" s="69">
-        <v>-16384</v>
-      </c>
-    </row>
-    <row r="39" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B39" s="70">
-        <v>8</v>
-      </c>
-      <c r="C39" s="70">
-        <v>-32767</v>
-      </c>
-      <c r="D39" s="70">
-        <v>2</v>
-      </c>
-      <c r="E39" s="70">
-        <v>-16384</v>
-      </c>
-    </row>
-    <row r="40" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B40" s="69">
-        <v>9</v>
-      </c>
-      <c r="C40" s="69">
-        <v>32767</v>
-      </c>
-      <c r="D40" s="69">
-        <v>-2</v>
-      </c>
-      <c r="E40" s="69">
-        <v>-16384</v>
-      </c>
-    </row>
-    <row r="41" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B41" s="50">
-        <v>10</v>
-      </c>
-      <c r="C41" s="50">
-        <v>7</v>
-      </c>
-      <c r="D41" s="50"/>
-      <c r="E41" s="50"/>
-    </row>
-    <row r="42" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B42" s="69">
-        <v>11</v>
-      </c>
-      <c r="C42" s="69"/>
-      <c r="D42" s="69">
-        <v>7</v>
-      </c>
-      <c r="E42" s="69"/>
-    </row>
-    <row r="43" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B43" s="50">
-        <v>12</v>
-      </c>
-      <c r="C43" s="50">
-        <v>-32768</v>
-      </c>
-      <c r="D43" s="50">
-        <v>-1</v>
-      </c>
-      <c r="E43" s="50">
-        <v>32768</v>
-      </c>
-    </row>
-    <row r="44" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B44" s="75"/>
-      <c r="C44" s="75"/>
-      <c r="D44" s="75"/>
-      <c r="E44" s="75"/>
-    </row>
-    <row r="47" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B47" s="79" t="s">
-        <v>327</v>
-      </c>
-      <c r="C47" s="79"/>
-      <c r="D47" s="79"/>
-      <c r="E47" s="79"/>
-    </row>
-    <row r="48" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B48" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C48" s="80"/>
-      <c r="D48" s="80"/>
-      <c r="E48" s="80"/>
-    </row>
-    <row r="50" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B50" s="78" t="s">
-        <v>328</v>
-      </c>
-      <c r="C50" s="78"/>
-      <c r="D50" s="78"/>
-      <c r="E50" s="78"/>
-    </row>
-    <row r="51" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B51" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C51" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D51" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E51" s="71" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B52" s="71" t="s">
-        <v>323</v>
-      </c>
-      <c r="C52" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D52" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E52" s="71" t="s">
-        <v>322</v>
       </c>
     </row>
     <row r="53" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B53" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C53" s="69">
         <v>7</v>
       </c>
       <c r="D53" s="69">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E53" s="69">
-        <v>2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="54" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B54" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C54" s="70">
         <v>-7</v>
       </c>
       <c r="D54" s="70">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E54" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="55" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B55" s="69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C55" s="69">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D55" s="69">
-        <v>-3</v>
+        <v>5</v>
       </c>
       <c r="E55" s="69">
-        <v>-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B56" s="70">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C56" s="70">
-        <v>-7</v>
+        <v>2147483647</v>
       </c>
       <c r="D56" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="E56" s="70">
-        <v>2</v>
+        <v>1073741823</v>
       </c>
     </row>
     <row r="57" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B57" s="69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C57" s="69">
-        <v>0</v>
+        <v>-2147483648</v>
       </c>
       <c r="D57" s="69">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E57" s="69">
-        <v>0</v>
+        <v>-1073741824</v>
       </c>
     </row>
     <row r="58" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B58" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C58" s="70">
-        <v>2147483647</v>
+        <v>-2147483647</v>
       </c>
       <c r="D58" s="70">
         <v>2</v>
       </c>
       <c r="E58" s="70">
-        <v>1073741823</v>
+        <v>-1073741824</v>
       </c>
     </row>
     <row r="59" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B59" s="69">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C59" s="69">
-        <v>-2147483648</v>
+        <v>2147483647</v>
       </c>
       <c r="D59" s="69">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="E59" s="69">
         <v>-1073741824</v>
       </c>
     </row>
     <row r="60" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B60" s="70">
-        <v>8</v>
-      </c>
-      <c r="C60" s="70">
-        <v>-2147483647</v>
-      </c>
-      <c r="D60" s="70">
-        <v>2</v>
-      </c>
-      <c r="E60" s="70">
-        <v>-1073741824</v>
-      </c>
+      <c r="B60" s="50">
+        <v>10</v>
+      </c>
+      <c r="C60" s="50">
+        <v>7</v>
+      </c>
+      <c r="D60" s="50"/>
+      <c r="E60" s="50"/>
     </row>
     <row r="61" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B61" s="69">
-        <v>9</v>
-      </c>
-      <c r="C61" s="69">
-        <v>2147483647</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="C61" s="69"/>
       <c r="D61" s="69">
-        <v>-2</v>
-      </c>
-      <c r="E61" s="69">
-        <v>-1073741824</v>
-      </c>
-    </row>
-    <row r="62" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B62" s="50">
-        <v>10</v>
-      </c>
-      <c r="C62" s="50">
         <v>7</v>
       </c>
-      <c r="D62" s="50"/>
-      <c r="E62" s="50"/>
-    </row>
-    <row r="63" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B63" s="69">
-        <v>11</v>
-      </c>
-      <c r="C63" s="69"/>
-      <c r="D63" s="69">
-        <v>7</v>
-      </c>
-      <c r="E63" s="69"/>
-    </row>
-    <row r="67" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B67" s="79" t="s">
+      <c r="E61" s="69"/>
+    </row>
+    <row r="65" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B65" s="84" t="s">
         <v>329</v>
       </c>
-      <c r="C67" s="79"/>
-      <c r="D67" s="79"/>
-      <c r="E67" s="79"/>
+      <c r="C65" s="84"/>
+      <c r="D65" s="84"/>
+      <c r="E65" s="84"/>
+    </row>
+    <row r="66" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B66" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C66" s="85"/>
+      <c r="D66" s="85"/>
+      <c r="E66" s="85"/>
     </row>
     <row r="68" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B68" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C68" s="80"/>
-      <c r="D68" s="80"/>
-      <c r="E68" s="80"/>
+      <c r="B68" s="86" t="s">
+        <v>330</v>
+      </c>
+      <c r="C68" s="86"/>
+      <c r="D68" s="86"/>
+      <c r="E68" s="86"/>
+    </row>
+    <row r="69" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B69" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C69" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D69" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E69" s="71" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="70" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B70" s="78" t="s">
-        <v>330</v>
-      </c>
-      <c r="C70" s="78"/>
-      <c r="D70" s="78"/>
-      <c r="E70" s="78"/>
+      <c r="B70" s="71" t="s">
+        <v>323</v>
+      </c>
+      <c r="C70" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D70" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E70" s="71" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="71" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B71" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C71" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D71" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E71" s="71" t="s">
-        <v>0</v>
+      <c r="B71" s="69">
+        <v>1</v>
+      </c>
+      <c r="C71" s="72" t="s">
+        <v>92</v>
+      </c>
+      <c r="D71" s="72" t="s">
+        <v>331</v>
+      </c>
+      <c r="E71" s="72" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="72" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B72" s="71" t="s">
-        <v>323</v>
-      </c>
-      <c r="C72" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D72" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E72" s="71" t="s">
-        <v>322</v>
+      <c r="B72" s="70">
+        <v>2</v>
+      </c>
+      <c r="C72" s="73" t="s">
+        <v>144</v>
+      </c>
+      <c r="D72" s="73" t="s">
+        <v>331</v>
+      </c>
+      <c r="E72" s="73" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="73" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B73" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C73" s="72" t="s">
         <v>92</v>
       </c>
       <c r="D73" s="72" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E73" s="72" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
     </row>
     <row r="74" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B74" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C74" s="73" t="s">
         <v>144</v>
       </c>
       <c r="D74" s="73" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E74" s="73" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="75" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B75" s="69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C75" s="72" t="s">
-        <v>92</v>
+        <v>24</v>
       </c>
       <c r="D75" s="72" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="E75" s="72" t="s">
-        <v>333</v>
+        <v>24</v>
       </c>
     </row>
     <row r="76" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B76" s="70">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C76" s="73" t="s">
-        <v>144</v>
+        <v>335</v>
       </c>
       <c r="D76" s="73" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E76" s="73" t="s">
-        <v>332</v>
+        <v>336</v>
       </c>
     </row>
     <row r="77" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B77" s="69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C77" s="72" t="s">
-        <v>24</v>
+        <v>337</v>
       </c>
       <c r="D77" s="72" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E77" s="72" t="s">
-        <v>24</v>
+        <v>338</v>
       </c>
     </row>
     <row r="78" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B78" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C78" s="73" t="s">
-        <v>335</v>
+        <v>339</v>
       </c>
       <c r="D78" s="73" t="s">
         <v>332</v>
       </c>
       <c r="E78" s="73" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
     </row>
     <row r="79" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B79" s="69">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C79" s="72" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="D79" s="72" t="s">
-        <v>332</v>
+        <v>63</v>
       </c>
       <c r="E79" s="72" t="s">
         <v>338</v>
       </c>
     </row>
     <row r="80" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B80" s="70">
-        <v>8</v>
-      </c>
-      <c r="C80" s="73" t="s">
-        <v>339</v>
-      </c>
-      <c r="D80" s="73" t="s">
-        <v>332</v>
-      </c>
-      <c r="E80" s="73" t="s">
-        <v>338</v>
-      </c>
+      <c r="B80" s="50">
+        <v>10</v>
+      </c>
+      <c r="C80" s="50">
+        <v>7</v>
+      </c>
+      <c r="D80" s="50"/>
+      <c r="E80" s="50"/>
     </row>
     <row r="81" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B81" s="69">
-        <v>9</v>
-      </c>
-      <c r="C81" s="72" t="s">
-        <v>335</v>
-      </c>
-      <c r="D81" s="72" t="s">
-        <v>63</v>
-      </c>
-      <c r="E81" s="72" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="82" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B82" s="50">
-        <v>10</v>
-      </c>
-      <c r="C82" s="50">
+        <v>11</v>
+      </c>
+      <c r="C81" s="69"/>
+      <c r="D81" s="69">
         <v>7</v>
       </c>
-      <c r="D82" s="50"/>
-      <c r="E82" s="50"/>
-    </row>
-    <row r="83" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B83" s="69">
-        <v>11</v>
-      </c>
-      <c r="C83" s="69"/>
-      <c r="D83" s="69">
+      <c r="E81" s="69"/>
+    </row>
+    <row r="85" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B85" s="84" t="s">
+        <v>343</v>
+      </c>
+      <c r="C85" s="84"/>
+      <c r="D85" s="84"/>
+      <c r="E85" s="84"/>
+    </row>
+    <row r="86" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B86" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C86" s="85"/>
+      <c r="D86" s="85"/>
+      <c r="E86" s="85"/>
+    </row>
+    <row r="88" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B88" s="86" t="s">
+        <v>342</v>
+      </c>
+      <c r="C88" s="86"/>
+      <c r="D88" s="86"/>
+      <c r="E88" s="86"/>
+    </row>
+    <row r="89" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B89" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C89" s="74" t="s">
+        <v>321</v>
+      </c>
+      <c r="D89" s="74" t="s">
+        <v>281</v>
+      </c>
+      <c r="E89" s="71" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="90" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B90" s="74" t="s">
+        <v>323</v>
+      </c>
+      <c r="C90" s="74" t="s">
+        <v>321</v>
+      </c>
+      <c r="D90" s="74" t="s">
+        <v>281</v>
+      </c>
+      <c r="E90" s="71" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="91" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B91" s="69">
+        <v>1</v>
+      </c>
+      <c r="C91" s="69">
         <v>7</v>
       </c>
-      <c r="E83" s="69"/>
-    </row>
-    <row r="87" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B87" s="79" t="s">
-        <v>343</v>
-      </c>
-      <c r="C87" s="79"/>
-      <c r="D87" s="79"/>
-      <c r="E87" s="79"/>
-    </row>
-    <row r="88" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B88" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C88" s="80"/>
-      <c r="D88" s="80"/>
-      <c r="E88" s="80"/>
-    </row>
-    <row r="90" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B90" s="78" t="s">
-        <v>342</v>
-      </c>
-      <c r="C90" s="78"/>
-      <c r="D90" s="78"/>
-      <c r="E90" s="78"/>
-    </row>
-    <row r="91" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B91" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C91" s="74" t="s">
-        <v>321</v>
-      </c>
-      <c r="D91" s="74" t="s">
-        <v>281</v>
-      </c>
-      <c r="E91" s="71" t="s">
-        <v>0</v>
+      <c r="D91" s="69">
+        <v>3</v>
+      </c>
+      <c r="E91" s="69">
+        <v>2</v>
       </c>
     </row>
     <row r="92" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B92" s="74" t="s">
-        <v>323</v>
-      </c>
-      <c r="C92" s="74" t="s">
-        <v>321</v>
-      </c>
-      <c r="D92" s="74" t="s">
-        <v>281</v>
-      </c>
-      <c r="E92" s="71" t="s">
-        <v>322</v>
+      <c r="B92" s="70">
+        <v>2</v>
+      </c>
+      <c r="C92" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D92" s="70">
+        <v>3</v>
+      </c>
+      <c r="E92" s="70">
+        <v>-3</v>
       </c>
     </row>
     <row r="93" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B93" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C93" s="69">
         <v>7</v>
       </c>
       <c r="D93" s="69">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E93" s="69">
-        <v>2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="94" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B94" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C94" s="70">
         <v>-7</v>
       </c>
       <c r="D94" s="70">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E94" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="95" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B95" s="69">
-        <v>3</v>
-      </c>
-      <c r="C95" s="69">
-        <v>7</v>
-      </c>
-      <c r="D95" s="69">
-        <v>-3</v>
+        <v>5</v>
+      </c>
+      <c r="C95" s="76" t="s">
+        <v>352</v>
+      </c>
+      <c r="D95" s="76" t="s">
+        <v>353</v>
       </c>
       <c r="E95" s="69">
-        <v>-3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="96" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B96" s="70">
-        <v>4</v>
-      </c>
-      <c r="C96" s="70">
-        <v>-7</v>
-      </c>
-      <c r="D96" s="70">
-        <v>-3</v>
+        <v>6</v>
+      </c>
+      <c r="C96" s="77" t="s">
+        <v>350</v>
+      </c>
+      <c r="D96" s="77" t="s">
+        <v>353</v>
       </c>
       <c r="E96" s="70">
-        <v>2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="97" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B97" s="69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C97" s="76" t="s">
         <v>352</v>
       </c>
       <c r="D97" s="76" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E97" s="69">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="98" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B98" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C98" s="77" t="s">
         <v>350</v>
       </c>
       <c r="D98" s="77" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E98" s="70">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="99" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B99" s="69">
+        <v>9</v>
+      </c>
+      <c r="C99" s="69">
+        <v>0</v>
+      </c>
+      <c r="D99" s="76" t="s">
+        <v>354</v>
+      </c>
+      <c r="E99" s="69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B100" s="50">
+        <v>10</v>
+      </c>
+      <c r="C100" s="50">
         <v>7</v>
       </c>
-      <c r="C99" s="76" t="s">
-        <v>352</v>
-      </c>
-      <c r="D99" s="76" t="s">
-        <v>351</v>
-      </c>
-      <c r="E99" s="69">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="100" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B100" s="70">
-        <v>8</v>
-      </c>
-      <c r="C100" s="77" t="s">
-        <v>350</v>
-      </c>
-      <c r="D100" s="77" t="s">
-        <v>351</v>
-      </c>
-      <c r="E100" s="70">
-        <v>1</v>
-      </c>
+      <c r="D100" s="50"/>
+      <c r="E100" s="50"/>
     </row>
     <row r="101" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B101" s="69">
-        <v>9</v>
-      </c>
-      <c r="C101" s="69">
-        <v>0</v>
-      </c>
-      <c r="D101" s="76" t="s">
-        <v>354</v>
-      </c>
-      <c r="E101" s="69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="102" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B102" s="50">
-        <v>10</v>
-      </c>
-      <c r="C102" s="50">
+        <v>11</v>
+      </c>
+      <c r="C101" s="69"/>
+      <c r="D101" s="69">
         <v>7</v>
       </c>
-      <c r="D102" s="50"/>
-      <c r="E102" s="50"/>
-    </row>
-    <row r="103" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B103" s="69">
-        <v>11</v>
-      </c>
-      <c r="C103" s="69"/>
-      <c r="D103" s="69">
+      <c r="E101" s="69"/>
+    </row>
+    <row r="105" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B105" s="84" t="s">
+        <v>344</v>
+      </c>
+      <c r="C105" s="84"/>
+      <c r="D105" s="84"/>
+      <c r="E105" s="84"/>
+    </row>
+    <row r="106" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B106" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C106" s="85"/>
+      <c r="D106" s="85"/>
+      <c r="E106" s="85"/>
+    </row>
+    <row r="108" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B108" s="86" t="s">
+        <v>345</v>
+      </c>
+      <c r="C108" s="86"/>
+      <c r="D108" s="86"/>
+      <c r="E108" s="86"/>
+    </row>
+    <row r="109" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B109" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C109" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D109" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E109" s="71" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="110" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B110" s="71" t="s">
+        <v>323</v>
+      </c>
+      <c r="C110" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D110" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E110" s="71" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="111" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B111" s="69">
+        <v>1</v>
+      </c>
+      <c r="C111" s="69">
         <v>7</v>
       </c>
-      <c r="E103" s="69"/>
-    </row>
-    <row r="107" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B107" s="79" t="s">
-        <v>344</v>
-      </c>
-      <c r="C107" s="79"/>
-      <c r="D107" s="79"/>
-      <c r="E107" s="79"/>
-    </row>
-    <row r="108" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B108" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C108" s="80"/>
-      <c r="D108" s="80"/>
-      <c r="E108" s="80"/>
-    </row>
-    <row r="110" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B110" s="78" t="s">
-        <v>345</v>
-      </c>
-      <c r="C110" s="78"/>
-      <c r="D110" s="78"/>
-      <c r="E110" s="78"/>
-    </row>
-    <row r="111" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B111" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C111" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D111" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E111" s="71" t="s">
-        <v>0</v>
+      <c r="D111" s="69">
+        <v>3</v>
+      </c>
+      <c r="E111" s="69">
+        <v>2</v>
       </c>
     </row>
     <row r="112" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B112" s="71" t="s">
-        <v>323</v>
-      </c>
-      <c r="C112" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D112" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E112" s="71" t="s">
-        <v>322</v>
+      <c r="B112" s="70">
+        <v>2</v>
+      </c>
+      <c r="C112" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D112" s="70">
+        <v>3</v>
+      </c>
+      <c r="E112" s="70">
+        <v>-3</v>
       </c>
     </row>
     <row r="113" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B113" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C113" s="69">
         <v>7</v>
       </c>
       <c r="D113" s="69">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E113" s="69">
-        <v>2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="114" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B114" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C114" s="70">
         <v>-7</v>
       </c>
       <c r="D114" s="70">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E114" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="115" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B115" s="69">
-        <v>3</v>
-      </c>
-      <c r="C115" s="69">
-        <v>7</v>
-      </c>
-      <c r="D115" s="69">
-        <v>-3</v>
+        <v>5</v>
+      </c>
+      <c r="C115" s="76" t="s">
+        <v>352</v>
+      </c>
+      <c r="D115" s="76" t="s">
+        <v>353</v>
       </c>
       <c r="E115" s="69">
-        <v>-3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="116" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B116" s="70">
-        <v>4</v>
-      </c>
-      <c r="C116" s="70">
-        <v>-7</v>
-      </c>
-      <c r="D116" s="70">
-        <v>-3</v>
+        <v>6</v>
+      </c>
+      <c r="C116" s="77" t="s">
+        <v>350</v>
+      </c>
+      <c r="D116" s="77" t="s">
+        <v>353</v>
       </c>
       <c r="E116" s="70">
-        <v>2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="117" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B117" s="69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C117" s="76" t="s">
         <v>352</v>
       </c>
       <c r="D117" s="76" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E117" s="69">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="118" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B118" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C118" s="77" t="s">
         <v>350</v>
       </c>
       <c r="D118" s="77" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E118" s="70">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="119" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B119" s="69">
+        <v>9</v>
+      </c>
+      <c r="C119" s="69">
+        <v>0</v>
+      </c>
+      <c r="D119" s="76" t="s">
+        <v>354</v>
+      </c>
+      <c r="E119" s="69">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="125" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B125" s="84" t="s">
+        <v>346</v>
+      </c>
+      <c r="C125" s="84"/>
+      <c r="D125" s="84"/>
+      <c r="E125" s="84"/>
+    </row>
+    <row r="126" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B126" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C126" s="85"/>
+      <c r="D126" s="85"/>
+      <c r="E126" s="85"/>
+    </row>
+    <row r="128" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B128" s="86" t="s">
+        <v>347</v>
+      </c>
+      <c r="C128" s="86"/>
+      <c r="D128" s="86"/>
+      <c r="E128" s="86"/>
+    </row>
+    <row r="129" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B129" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C129" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D129" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E129" s="71" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="130" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B130" s="71" t="s">
+        <v>323</v>
+      </c>
+      <c r="C130" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D130" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E130" s="71" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="131" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B131" s="69">
+        <v>1</v>
+      </c>
+      <c r="C131" s="69">
         <v>7</v>
       </c>
-      <c r="C119" s="76" t="s">
-        <v>352</v>
-      </c>
-      <c r="D119" s="76" t="s">
-        <v>351</v>
-      </c>
-      <c r="E119" s="69">
-        <v>-2</v>
-      </c>
-    </row>
-    <row r="120" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B120" s="70">
-        <v>8</v>
-      </c>
-      <c r="C120" s="77" t="s">
-        <v>350</v>
-      </c>
-      <c r="D120" s="77" t="s">
-        <v>351</v>
-      </c>
-      <c r="E120" s="70">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="121" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B121" s="69">
-        <v>9</v>
-      </c>
-      <c r="C121" s="69">
-        <v>0</v>
-      </c>
-      <c r="D121" s="76" t="s">
-        <v>354</v>
-      </c>
-      <c r="E121" s="69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="127" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B127" s="79" t="s">
-        <v>346</v>
-      </c>
-      <c r="C127" s="79"/>
-      <c r="D127" s="79"/>
-      <c r="E127" s="79"/>
-    </row>
-    <row r="128" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B128" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C128" s="80"/>
-      <c r="D128" s="80"/>
-      <c r="E128" s="80"/>
-    </row>
-    <row r="130" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B130" s="78" t="s">
-        <v>347</v>
-      </c>
-      <c r="C130" s="78"/>
-      <c r="D130" s="78"/>
-      <c r="E130" s="78"/>
-    </row>
-    <row r="131" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B131" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C131" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D131" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E131" s="71" t="s">
-        <v>0</v>
+      <c r="D131" s="69">
+        <v>3</v>
+      </c>
+      <c r="E131" s="69">
+        <v>2</v>
       </c>
     </row>
     <row r="132" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B132" s="71" t="s">
-        <v>323</v>
-      </c>
-      <c r="C132" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D132" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E132" s="71" t="s">
-        <v>322</v>
+      <c r="B132" s="70">
+        <v>2</v>
+      </c>
+      <c r="C132" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D132" s="70">
+        <v>3</v>
+      </c>
+      <c r="E132" s="70">
+        <v>-3</v>
       </c>
     </row>
     <row r="133" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B133" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C133" s="69">
         <v>7</v>
       </c>
       <c r="D133" s="69">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E133" s="69">
-        <v>2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="134" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B134" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C134" s="70">
         <v>-7</v>
       </c>
       <c r="D134" s="70">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E134" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="135" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B135" s="69">
-        <v>3</v>
-      </c>
-      <c r="C135" s="69">
-        <v>7</v>
-      </c>
-      <c r="D135" s="69">
-        <v>-3</v>
+        <v>5</v>
+      </c>
+      <c r="C135" s="76" t="s">
+        <v>352</v>
+      </c>
+      <c r="D135" s="76" t="s">
+        <v>353</v>
       </c>
       <c r="E135" s="69">
-        <v>-3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B136" s="70">
-        <v>4</v>
-      </c>
-      <c r="C136" s="70">
-        <v>-7</v>
-      </c>
-      <c r="D136" s="70">
-        <v>-3</v>
+        <v>6</v>
+      </c>
+      <c r="C136" s="77" t="s">
+        <v>350</v>
+      </c>
+      <c r="D136" s="77" t="s">
+        <v>353</v>
       </c>
       <c r="E136" s="70">
-        <v>2</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="137" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B137" s="69">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C137" s="76" t="s">
         <v>352</v>
       </c>
       <c r="D137" s="76" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E137" s="69">
-        <v>1</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="138" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B138" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C138" s="77" t="s">
         <v>350</v>
       </c>
       <c r="D138" s="77" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="E138" s="70">
-        <v>-2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B139" s="69">
-        <v>7</v>
-      </c>
-      <c r="C139" s="76" t="s">
-        <v>352</v>
+        <v>9</v>
+      </c>
+      <c r="C139" s="69">
+        <v>0</v>
       </c>
       <c r="D139" s="76" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="E139" s="69">
-        <v>-2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="140" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B140" s="70">
-        <v>8</v>
-      </c>
-      <c r="C140" s="77" t="s">
-        <v>350</v>
-      </c>
-      <c r="D140" s="77" t="s">
-        <v>351</v>
-      </c>
-      <c r="E140" s="70">
-        <v>1</v>
+        <v>10</v>
+      </c>
+      <c r="C140" s="73" t="s">
+        <v>355</v>
+      </c>
+      <c r="D140" s="73">
+        <v>97</v>
+      </c>
+      <c r="E140" s="73" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="141" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B141" s="69">
-        <v>9</v>
-      </c>
-      <c r="C141" s="69">
-        <v>0</v>
-      </c>
-      <c r="D141" s="76" t="s">
-        <v>354</v>
-      </c>
-      <c r="E141" s="69">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="142" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B142" s="70">
-        <v>10</v>
-      </c>
-      <c r="C142" s="73" t="s">
-        <v>355</v>
-      </c>
-      <c r="D142" s="73">
+        <v>11</v>
+      </c>
+      <c r="C141" s="72" t="s">
+        <v>356</v>
+      </c>
+      <c r="D141" s="72">
         <v>97</v>
       </c>
-      <c r="E142" s="73" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="143" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B143" s="69">
-        <v>11</v>
-      </c>
-      <c r="C143" s="72" t="s">
-        <v>356</v>
-      </c>
-      <c r="D143" s="72">
-        <v>97</v>
-      </c>
-      <c r="E143" s="72" t="s">
+      <c r="E141" s="72" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="147" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B147" s="79" t="s">
+    <row r="145" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B145" s="84" t="s">
         <v>348</v>
       </c>
-      <c r="C147" s="79"/>
-      <c r="D147" s="79"/>
-      <c r="E147" s="79"/>
+      <c r="C145" s="84"/>
+      <c r="D145" s="84"/>
+      <c r="E145" s="84"/>
+    </row>
+    <row r="146" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B146" s="85" t="s">
+        <v>324</v>
+      </c>
+      <c r="C146" s="85"/>
+      <c r="D146" s="85"/>
+      <c r="E146" s="85"/>
     </row>
     <row r="148" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B148" s="80" t="s">
-        <v>324</v>
-      </c>
-      <c r="C148" s="80"/>
-      <c r="D148" s="80"/>
-      <c r="E148" s="80"/>
+      <c r="B148" s="86" t="s">
+        <v>349</v>
+      </c>
+      <c r="C148" s="86"/>
+      <c r="D148" s="86"/>
+      <c r="E148" s="86"/>
+    </row>
+    <row r="149" spans="2:5" x14ac:dyDescent="0.15">
+      <c r="B149" s="71" t="s">
+        <v>316</v>
+      </c>
+      <c r="C149" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D149" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E149" s="71" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="150" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B150" s="78" t="s">
-        <v>349</v>
-      </c>
-      <c r="C150" s="78"/>
-      <c r="D150" s="78"/>
-      <c r="E150" s="78"/>
+      <c r="B150" s="71" t="s">
+        <v>323</v>
+      </c>
+      <c r="C150" s="71" t="s">
+        <v>321</v>
+      </c>
+      <c r="D150" s="71" t="s">
+        <v>281</v>
+      </c>
+      <c r="E150" s="71" t="s">
+        <v>322</v>
+      </c>
     </row>
     <row r="151" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B151" s="71" t="s">
-        <v>316</v>
-      </c>
-      <c r="C151" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D151" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E151" s="71" t="s">
-        <v>0</v>
+      <c r="B151" s="69">
+        <v>1</v>
+      </c>
+      <c r="C151" s="69">
+        <v>7</v>
+      </c>
+      <c r="D151" s="69">
+        <v>3</v>
+      </c>
+      <c r="E151" s="69">
+        <v>2</v>
       </c>
     </row>
     <row r="152" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B152" s="71" t="s">
-        <v>323</v>
-      </c>
-      <c r="C152" s="71" t="s">
-        <v>321</v>
-      </c>
-      <c r="D152" s="71" t="s">
-        <v>281</v>
-      </c>
-      <c r="E152" s="71" t="s">
-        <v>322</v>
+      <c r="B152" s="70">
+        <v>2</v>
+      </c>
+      <c r="C152" s="70">
+        <v>-7</v>
+      </c>
+      <c r="D152" s="70">
+        <v>3</v>
+      </c>
+      <c r="E152" s="70">
+        <v>-3</v>
       </c>
     </row>
     <row r="153" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B153" s="69">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C153" s="69">
         <v>7</v>
       </c>
       <c r="D153" s="69">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E153" s="69">
-        <v>2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="154" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B154" s="70">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C154" s="70">
         <v>-7</v>
       </c>
       <c r="D154" s="70">
-        <v>3</v>
+        <v>-3</v>
       </c>
       <c r="E154" s="70">
-        <v>-3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="155" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B155" s="69">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C155" s="69">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="D155" s="69">
-        <v>-3</v>
+        <v>97</v>
       </c>
       <c r="E155" s="69">
-        <v>-3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="156" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B156" s="70">
-        <v>4</v>
-      </c>
-      <c r="C156" s="70">
-        <v>-7</v>
-      </c>
-      <c r="D156" s="70">
-        <v>-3</v>
-      </c>
-      <c r="E156" s="70">
-        <v>2</v>
+        <v>6</v>
+      </c>
+      <c r="C156" s="73" t="s">
+        <v>355</v>
+      </c>
+      <c r="D156" s="73">
+        <v>97</v>
+      </c>
+      <c r="E156" s="73" t="s">
+        <v>357</v>
       </c>
     </row>
     <row r="157" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B157" s="69">
-        <v>5</v>
-      </c>
-      <c r="C157" s="69">
-        <v>0</v>
-      </c>
-      <c r="D157" s="69">
+        <v>7</v>
+      </c>
+      <c r="C157" s="72" t="s">
+        <v>356</v>
+      </c>
+      <c r="D157" s="72">
         <v>97</v>
       </c>
-      <c r="E157" s="69">
-        <v>0</v>
+      <c r="E157" s="72" t="s">
+        <v>358</v>
       </c>
     </row>
     <row r="158" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B158" s="70">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C158" s="73" t="s">
         <v>355</v>
       </c>
       <c r="D158" s="73">
-        <v>97</v>
+        <v>-97</v>
       </c>
       <c r="E158" s="73" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
     </row>
     <row r="159" spans="2:5" x14ac:dyDescent="0.15">
       <c r="B159" s="69">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C159" s="72" t="s">
         <v>356</v>
       </c>
       <c r="D159" s="72">
-        <v>97</v>
+        <v>-97</v>
       </c>
       <c r="E159" s="72" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="160" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B160" s="70">
-        <v>8</v>
-      </c>
-      <c r="C160" s="73" t="s">
-        <v>355</v>
-      </c>
-      <c r="D160" s="73">
-        <v>-97</v>
-      </c>
-      <c r="E160" s="73" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="161" spans="2:5" x14ac:dyDescent="0.15">
-      <c r="B161" s="69">
-        <v>9</v>
-      </c>
-      <c r="C161" s="72" t="s">
-        <v>356</v>
-      </c>
-      <c r="D161" s="72">
-        <v>-97</v>
-      </c>
-      <c r="E161" s="72" t="s">
         <v>357</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="24">
+    <mergeCell ref="B128:E128"/>
+    <mergeCell ref="B145:E145"/>
+    <mergeCell ref="B146:E146"/>
+    <mergeCell ref="B148:E148"/>
+    <mergeCell ref="B105:E105"/>
+    <mergeCell ref="B106:E106"/>
+    <mergeCell ref="B108:E108"/>
+    <mergeCell ref="B125:E125"/>
+    <mergeCell ref="B126:E126"/>
+    <mergeCell ref="B66:E66"/>
+    <mergeCell ref="B68:E68"/>
+    <mergeCell ref="B85:E85"/>
+    <mergeCell ref="B86:E86"/>
+    <mergeCell ref="B88:E88"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B45:E45"/>
+    <mergeCell ref="B46:E46"/>
+    <mergeCell ref="B48:E48"/>
+    <mergeCell ref="B65:E65"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="B6:E6"/>
     <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B25:E25"/>
     <mergeCell ref="B26:E26"/>
-    <mergeCell ref="B27:E27"/>
-    <mergeCell ref="B29:E29"/>
-    <mergeCell ref="B47:E47"/>
-    <mergeCell ref="B48:E48"/>
-    <mergeCell ref="B50:E50"/>
-    <mergeCell ref="B67:E67"/>
-    <mergeCell ref="B68:E68"/>
-    <mergeCell ref="B70:E70"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:E88"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="B130:E130"/>
-    <mergeCell ref="B147:E147"/>
-    <mergeCell ref="B148:E148"/>
-    <mergeCell ref="B150:E150"/>
-    <mergeCell ref="B107:E107"/>
-    <mergeCell ref="B108:E108"/>
-    <mergeCell ref="B110:E110"/>
-    <mergeCell ref="B127:E127"/>
-    <mergeCell ref="B128:E128"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -10761,22 +10733,22 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:3" ht="14" x14ac:dyDescent="0.15">
-      <c r="B2" s="92" t="s">
+      <c r="B2" s="100" t="s">
         <v>269</v>
       </c>
-      <c r="C2" s="92"/>
+      <c r="C2" s="100"/>
     </row>
     <row r="3" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B3" s="93" t="s">
+      <c r="B3" s="92" t="s">
         <v>270</v>
       </c>
-      <c r="C3" s="93"/>
+      <c r="C3" s="92"/>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B5" s="94" t="s">
+      <c r="B5" s="93" t="s">
         <v>271</v>
       </c>
-      <c r="C5" s="95"/>
+      <c r="C5" s="94"/>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B6" s="58" t="s">
@@ -10867,22 +10839,22 @@
       </c>
     </row>
     <row r="20" spans="2:3" ht="14" x14ac:dyDescent="0.15">
-      <c r="B20" s="92" t="s">
+      <c r="B20" s="100" t="s">
         <v>169</v>
       </c>
-      <c r="C20" s="92"/>
+      <c r="C20" s="100"/>
     </row>
     <row r="21" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B21" s="93" t="s">
+      <c r="B21" s="92" t="s">
         <v>170</v>
       </c>
-      <c r="C21" s="93"/>
+      <c r="C21" s="92"/>
     </row>
     <row r="23" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B23" s="94" t="s">
+      <c r="B23" s="93" t="s">
         <v>171</v>
       </c>
-      <c r="C23" s="95"/>
+      <c r="C23" s="94"/>
     </row>
     <row r="24" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B24" s="58" t="s">
@@ -10973,22 +10945,22 @@
       </c>
     </row>
     <row r="38" spans="2:3" ht="14" x14ac:dyDescent="0.15">
-      <c r="B38" s="92" t="s">
+      <c r="B38" s="100" t="s">
         <v>107</v>
       </c>
-      <c r="C38" s="92"/>
+      <c r="C38" s="100"/>
     </row>
     <row r="39" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B39" s="93" t="s">
+      <c r="B39" s="92" t="s">
         <v>108</v>
       </c>
-      <c r="C39" s="93"/>
+      <c r="C39" s="92"/>
     </row>
     <row r="41" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B41" s="94" t="s">
+      <c r="B41" s="93" t="s">
         <v>109</v>
       </c>
-      <c r="C41" s="95"/>
+      <c r="C41" s="94"/>
     </row>
     <row r="42" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B42" s="58" t="s">
@@ -11079,22 +11051,22 @@
       </c>
     </row>
     <row r="56" spans="2:3" ht="14" x14ac:dyDescent="0.15">
-      <c r="B56" s="92" t="s">
+      <c r="B56" s="100" t="s">
         <v>203</v>
       </c>
-      <c r="C56" s="92"/>
+      <c r="C56" s="100"/>
     </row>
     <row r="57" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B57" s="93" t="s">
+      <c r="B57" s="92" t="s">
         <v>204</v>
       </c>
-      <c r="C57" s="93"/>
+      <c r="C57" s="92"/>
     </row>
     <row r="59" spans="2:3" x14ac:dyDescent="0.15">
-      <c r="B59" s="94" t="s">
+      <c r="B59" s="93" t="s">
         <v>205</v>
       </c>
-      <c r="C59" s="95"/>
+      <c r="C59" s="94"/>
     </row>
     <row r="60" spans="2:3" x14ac:dyDescent="0.15">
       <c r="B60" s="58" t="s">
@@ -11185,31 +11157,31 @@
       </c>
     </row>
     <row r="74" spans="2:6" ht="14" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B74" s="81" t="s">
+      <c r="B74" s="78" t="s">
         <v>273</v>
       </c>
-      <c r="C74" s="82"/>
-      <c r="D74" s="82"/>
-      <c r="E74" s="82"/>
-      <c r="F74" s="82"/>
+      <c r="C74" s="79"/>
+      <c r="D74" s="79"/>
+      <c r="E74" s="79"/>
+      <c r="F74" s="79"/>
     </row>
     <row r="75" spans="2:6" ht="13" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="B75" s="96" t="s">
+      <c r="B75" s="95" t="s">
         <v>274</v>
       </c>
-      <c r="C75" s="97"/>
-      <c r="D75" s="97"/>
-      <c r="E75" s="97"/>
-      <c r="F75" s="97"/>
+      <c r="C75" s="96"/>
+      <c r="D75" s="96"/>
+      <c r="E75" s="96"/>
+      <c r="F75" s="96"/>
     </row>
     <row r="77" spans="2:6" x14ac:dyDescent="0.15">
-      <c r="B77" s="98" t="s">
+      <c r="B77" s="97" t="s">
         <v>272</v>
       </c>
-      <c r="C77" s="99"/>
-      <c r="D77" s="99"/>
-      <c r="E77" s="99"/>
-      <c r="F77" s="100"/>
+      <c r="C77" s="98"/>
+      <c r="D77" s="98"/>
+      <c r="E77" s="98"/>
+      <c r="F77" s="99"/>
     </row>
     <row r="78" spans="2:6" x14ac:dyDescent="0.15">
       <c r="B78" s="59" t="s">
@@ -11579,21 +11551,21 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B56:C56"/>
     <mergeCell ref="B57:C57"/>
     <mergeCell ref="B59:C59"/>
     <mergeCell ref="B74:F74"/>
     <mergeCell ref="B75:F75"/>
     <mergeCell ref="B77:F77"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="B56:C56"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="B21:C21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>